<commit_message>
feat: Enhance quiz import functionality with validation and helper services
</commit_message>
<xml_diff>
--- a/repo-learning-path/test-data/learning-path-import-full-test.xlsx
+++ b/repo-learning-path/test-data/learning-path-import-full-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DO_AN\BE_LMS\repo-learning-path\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBDF6C4-9376-4DD3-98AF-3806552F6140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F4D170E-4979-4DAE-85C0-1F0C307A22D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="466">
   <si>
     <t>PackageName</t>
   </si>
@@ -1155,72 +1155,6 @@
     <t>Học phát âm theo lộ trình học</t>
   </si>
   <si>
-    <t>Ngọn núi</t>
-  </si>
-  <si>
-    <t>Mặt trăng</t>
-  </si>
-  <si>
-    <t>Chữ "日" (Nhật) có nghĩa là gì?</t>
-  </si>
-  <si>
-    <t>Trắc nghiệm Hán tự cơ bản</t>
-  </si>
-  <si>
-    <t>Chữ Hán Nhập Môn</t>
-  </si>
-  <si>
-    <t>Khóa học nguồn gốc chữ Hán</t>
-  </si>
-  <si>
-    <t>Tiết 1</t>
-  </si>
-  <si>
-    <t>Luyện tập bộ thủ</t>
-  </si>
-  <si>
-    <t>Dữ liệu câu hỏi trắc nghiệm</t>
-  </si>
-  <si>
-    <t>Kiểm tra ý nghĩa Nhật Nguyệt Sơn Thủy</t>
-  </si>
-  <si>
-    <t>Trắc nghiệm Bộ Thủ</t>
-  </si>
-  <si>
-    <t>Bài kiểm tra tính điểm</t>
-  </si>
-  <si>
-    <t>Hình ảnh mặt trời</t>
-  </si>
-  <si>
-    <t>Con sông</t>
-  </si>
-  <si>
-    <t>Chữ nào sau đây có nghĩa là "Mặt trăng"?</t>
-  </si>
-  <si>
-    <t>Hình ảnh trăng khuyết</t>
-  </si>
-  <si>
-    <t>Cách phát âm của chữ "山" (Sơn) là gì?</t>
-  </si>
-  <si>
-    <t>Âm đọc ngọn núi</t>
-  </si>
-  <si>
-    <t>Trong các âm sau, âm nào là âm bật hơi?</t>
-  </si>
-  <si>
-    <t>Phát âm chữ p</t>
-  </si>
-  <si>
-    <t>Gói Trắc nghiệm lộ trình học</t>
-  </si>
-  <si>
-    <t>StudySetDesc</t>
-  </si>
-  <si>
     <t>Chinh Phục Tiếng Trung Sơ Cấp</t>
   </si>
   <si>
@@ -1312,6 +1246,183 @@
   </si>
   <si>
     <t>[{"char":"吃"},{"char":"饭"}]</t>
+  </si>
+  <si>
+    <t>Goi Trac nghiem tieng Trung co ban</t>
+  </si>
+  <si>
+    <t>Bo cau hoi tong hop cho ngu am, tu vung va ngu phap</t>
+  </si>
+  <si>
+    <t>Tieng Trung Nhap Mon</t>
+  </si>
+  <si>
+    <t>Hoc phat am pinyin va tu vung HSK 1</t>
+  </si>
+  <si>
+    <t>Tiet 1</t>
+  </si>
+  <si>
+    <t>On tap thanh mau va van mau</t>
+  </si>
+  <si>
+    <t>Thu muc Tu vung va Ngu am</t>
+  </si>
+  <si>
+    <t>Du lieu cau hoi trac nghiem va dien khuyet</t>
+  </si>
+  <si>
+    <t>Chu de Chao hoi va Gioi thieu</t>
+  </si>
+  <si>
+    <t>Kiem tra pinyin va tu vung co ban</t>
+  </si>
+  <si>
+    <t>Quiz 10 cau ve pinyin, nghia tu va mau cau don gian</t>
+  </si>
+  <si>
+    <t>900</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>Tu nao co nghia la xin chao trong tieng Trung?</t>
+  </si>
+  <si>
+    <t>Ni hao la loi chao pho bien</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>谢谢</t>
+  </si>
+  <si>
+    <t>FALSE</t>
+  </si>
+  <si>
+    <t>对不起</t>
+  </si>
+  <si>
+    <t>Am nao la thanh 3 trong pinyin cua ma?</t>
+  </si>
+  <si>
+    <t>Thanh 3 co dang ha-xuong-roi len</t>
+  </si>
+  <si>
+    <t>má</t>
+  </si>
+  <si>
+    <t>mǎ</t>
+  </si>
+  <si>
+    <t>mà</t>
+  </si>
+  <si>
+    <t>FILL_IN_BLANK</t>
+  </si>
+  <si>
+    <t>Dien vao cho trong de hoan thanh cau: Wo ___ Zhongguo ren.</t>
+  </si>
+  <si>
+    <t>Dong tu 'shi' dung de noi 'la'</t>
+  </si>
+  <si>
+    <t>Wo ___ Zhongguo ren.</t>
+  </si>
+  <si>
+    <t>TYPE</t>
+  </si>
+  <si>
+    <t>shi</t>
+  </si>
+  <si>
+    <t>Shi|shi</t>
+  </si>
+  <si>
+    <t>Dong tu to be</t>
+  </si>
+  <si>
+    <t>MATCHING_PAIRS</t>
+  </si>
+  <si>
+    <t>Noi tu tieng Trung voi nghia tieng Viet</t>
+  </si>
+  <si>
+    <t>Ghep dung 4 cap tu</t>
+  </si>
+  <si>
+    <t>xue sheng</t>
+  </si>
+  <si>
+    <t>hoc sinh</t>
+  </si>
+  <si>
+    <t>lao shi</t>
+  </si>
+  <si>
+    <t>giao vien</t>
+  </si>
+  <si>
+    <t>学生</t>
+  </si>
+  <si>
+    <t>ban be</t>
+  </si>
+  <si>
+    <t>老师</t>
+  </si>
+  <si>
+    <t>gia dinh</t>
+  </si>
+  <si>
+    <t>SENTENCE_BUILDER</t>
+  </si>
+  <si>
+    <t>Sap xep tu de tao cau dung</t>
+  </si>
+  <si>
+    <t>Mau cau gioi thieu quoc tich</t>
+  </si>
+  <si>
+    <t>HARD</t>
+  </si>
+  <si>
+    <t>朋友</t>
+  </si>
+  <si>
+    <t>Toi la nguoi Viet Nam</t>
+  </si>
+  <si>
+    <t>Wo</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>家</t>
+  </si>
+  <si>
+    <t>Yuenan</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>ren</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>ma</t>
+  </si>
+  <si>
+    <t>4</t>
   </si>
 </sst>
 </file>
@@ -1739,40 +1850,40 @@
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>398</v>
+        <v>376</v>
       </c>
       <c r="B2" t="s">
-        <v>399</v>
+        <v>377</v>
       </c>
       <c r="C2" t="s">
-        <v>400</v>
+        <v>378</v>
       </c>
       <c r="D2" t="s">
-        <v>401</v>
+        <v>379</v>
       </c>
       <c r="E2" t="s">
-        <v>402</v>
+        <v>380</v>
       </c>
       <c r="F2" t="s">
-        <v>403</v>
+        <v>381</v>
       </c>
       <c r="G2" t="s">
-        <v>404</v>
+        <v>382</v>
       </c>
       <c r="H2" t="s">
-        <v>405</v>
+        <v>383</v>
       </c>
       <c r="I2" t="s">
-        <v>406</v>
+        <v>384</v>
       </c>
       <c r="J2" t="s">
-        <v>407</v>
+        <v>385</v>
       </c>
       <c r="K2">
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>408</v>
+        <v>386</v>
       </c>
       <c r="M2" t="s">
         <v>16</v>
@@ -1789,16 +1900,16 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="I3" t="s">
-        <v>409</v>
+        <v>387</v>
       </c>
       <c r="J3" t="s">
-        <v>410</v>
+        <v>388</v>
       </c>
       <c r="K3">
         <v>2</v>
       </c>
       <c r="L3" t="s">
-        <v>411</v>
+        <v>389</v>
       </c>
       <c r="M3" t="s">
         <v>18</v>
@@ -1815,16 +1926,16 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="I4" t="s">
-        <v>412</v>
+        <v>390</v>
       </c>
       <c r="J4" t="s">
-        <v>413</v>
+        <v>391</v>
       </c>
       <c r="K4">
         <v>3</v>
       </c>
       <c r="L4" t="s">
-        <v>414</v>
+        <v>392</v>
       </c>
       <c r="M4" t="s">
         <v>20</v>
@@ -1841,34 +1952,34 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
-        <v>415</v>
+        <v>393</v>
       </c>
       <c r="D5" t="s">
-        <v>416</v>
+        <v>394</v>
       </c>
       <c r="E5" t="s">
-        <v>417</v>
+        <v>395</v>
       </c>
       <c r="F5" t="s">
-        <v>418</v>
+        <v>396</v>
       </c>
       <c r="G5" t="s">
-        <v>419</v>
+        <v>397</v>
       </c>
       <c r="H5" t="s">
-        <v>420</v>
+        <v>398</v>
       </c>
       <c r="I5" t="s">
-        <v>421</v>
+        <v>399</v>
       </c>
       <c r="J5" t="s">
-        <v>422</v>
+        <v>400</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
       <c r="L5" t="s">
-        <v>423</v>
+        <v>401</v>
       </c>
       <c r="M5" t="s">
         <v>22</v>
@@ -1885,16 +1996,16 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="I6" t="s">
-        <v>424</v>
+        <v>402</v>
       </c>
       <c r="J6" t="s">
-        <v>425</v>
+        <v>403</v>
       </c>
       <c r="K6">
         <v>2</v>
       </c>
       <c r="L6" t="s">
-        <v>426</v>
+        <v>404</v>
       </c>
       <c r="M6" t="s">
         <v>24</v>
@@ -2610,7 +2721,7 @@
         <v>212</v>
       </c>
       <c r="Z6" t="s">
-        <v>428</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -3163,7 +3274,7 @@
         <v>301</v>
       </c>
       <c r="AJ6" t="s">
-        <v>427</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>
@@ -3548,7 +3659,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:AA17"/>
+  <dimension ref="A1:AB20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" bestFit="1" customWidth="1"/>
@@ -3562,23 +3673,23 @@
     <col min="9" max="9" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" customWidth="1"/>
-    <col min="13" max="13" width="32.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="28.88671875" customWidth="1"/>
-    <col min="20" max="20" width="26.44140625" customWidth="1"/>
-    <col min="21" max="21" width="10.44140625" customWidth="1"/>
-    <col min="22" max="22" width="18.88671875" customWidth="1"/>
-    <col min="23" max="23" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="25" max="27" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="16.88671875" customWidth="1"/>
+    <col min="14" max="14" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="28.88671875" customWidth="1"/>
+    <col min="21" max="21" width="26.44140625" customWidth="1"/>
+    <col min="22" max="22" width="10.44140625" customWidth="1"/>
+    <col min="23" max="23" width="18.88671875" customWidth="1"/>
+    <col min="24" max="24" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="26" max="28" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3613,7 +3724,7 @@
         <v>4</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>397</v>
+        <v>5</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>88</v>
@@ -3660,244 +3771,311 @@
       <c r="AA1" s="1" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="AB1" s="1"/>
+    </row>
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>396</v>
+        <v>407</v>
       </c>
       <c r="B2" t="s">
-        <v>379</v>
+        <v>408</v>
       </c>
       <c r="C2" t="s">
-        <v>380</v>
+        <v>409</v>
       </c>
       <c r="D2" t="s">
-        <v>218</v>
+        <v>147</v>
       </c>
       <c r="E2" t="s">
-        <v>381</v>
+        <v>410</v>
       </c>
       <c r="F2" t="s">
-        <v>382</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
+        <v>411</v>
+      </c>
+      <c r="G2" t="s">
+        <v>48</v>
       </c>
       <c r="H2" t="s">
-        <v>383</v>
+        <v>412</v>
       </c>
       <c r="I2" t="s">
-        <v>222</v>
+        <v>413</v>
       </c>
       <c r="J2" t="s">
-        <v>384</v>
+        <v>414</v>
       </c>
       <c r="K2" t="s">
-        <v>224</v>
-      </c>
-      <c r="L2" t="s">
-        <v>385</v>
+        <v>415</v>
       </c>
       <c r="M2" t="s">
-        <v>386</v>
+        <v>416</v>
       </c>
       <c r="N2" t="s">
-        <v>387</v>
+        <v>417</v>
       </c>
       <c r="O2" t="s">
         <v>105</v>
       </c>
-      <c r="P2">
-        <v>600</v>
-      </c>
-      <c r="Q2">
-        <v>80</v>
+      <c r="P2" t="s">
+        <v>418</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>419</v>
       </c>
       <c r="R2" t="s">
         <v>104</v>
       </c>
       <c r="S2" t="s">
-        <v>378</v>
+        <v>420</v>
       </c>
       <c r="T2" t="s">
-        <v>388</v>
-      </c>
-      <c r="U2">
-        <v>10</v>
+        <v>421</v>
+      </c>
+      <c r="U2" t="s">
+        <v>422</v>
       </c>
       <c r="V2" t="s">
         <v>105</v>
       </c>
       <c r="W2" t="s">
-        <v>240</v>
-      </c>
-      <c r="X2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+      <c r="X2" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="W3" t="s">
-        <v>377</v>
-      </c>
-      <c r="X3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+        <v>424</v>
+      </c>
+      <c r="X3" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="W4" t="s">
-        <v>376</v>
-      </c>
-      <c r="X4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+      <c r="X4" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="W5" t="s">
-        <v>389</v>
-      </c>
-      <c r="X5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+        <v>426</v>
+      </c>
+      <c r="X5" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="R6" t="s">
         <v>104</v>
       </c>
       <c r="S6" t="s">
-        <v>390</v>
+        <v>427</v>
       </c>
       <c r="T6" t="s">
-        <v>391</v>
-      </c>
-      <c r="U6">
-        <v>10</v>
+        <v>428</v>
+      </c>
+      <c r="U6" t="s">
+        <v>422</v>
       </c>
       <c r="V6" t="s">
         <v>105</v>
       </c>
       <c r="W6" t="s">
-        <v>75</v>
-      </c>
-      <c r="X6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+        <v>352</v>
+      </c>
+      <c r="X6" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="W7" t="s">
-        <v>242</v>
-      </c>
-      <c r="X7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+        <v>429</v>
+      </c>
+      <c r="X7" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="W8" t="s">
-        <v>261</v>
-      </c>
-      <c r="X8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+        <v>430</v>
+      </c>
+      <c r="X8" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="W9" t="s">
-        <v>283</v>
-      </c>
-      <c r="X9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+      <c r="X9" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="R10" t="s">
-        <v>104</v>
+        <v>432</v>
       </c>
       <c r="S10" t="s">
-        <v>392</v>
+        <v>433</v>
       </c>
       <c r="T10" t="s">
-        <v>393</v>
-      </c>
-      <c r="U10">
-        <v>10</v>
+        <v>434</v>
+      </c>
+      <c r="U10" t="s">
+        <v>422</v>
       </c>
       <c r="V10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="W10" t="s">
-        <v>263</v>
-      </c>
-      <c r="X10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+        <v>435</v>
+      </c>
+      <c r="X10" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="W11" t="s">
-        <v>285</v>
-      </c>
-      <c r="X11" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+        <v>437</v>
+      </c>
+      <c r="X11" t="s">
+        <v>438</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="R12" t="s">
+        <v>440</v>
+      </c>
+      <c r="S12" t="s">
+        <v>441</v>
+      </c>
+      <c r="T12" t="s">
+        <v>442</v>
+      </c>
+      <c r="U12" t="s">
+        <v>422</v>
+      </c>
+      <c r="V12" t="s">
+        <v>103</v>
+      </c>
       <c r="W12" t="s">
-        <v>227</v>
-      </c>
-      <c r="X12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+      <c r="X12" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="W13" t="s">
-        <v>244</v>
-      </c>
-      <c r="X13" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="R14" t="s">
-        <v>104</v>
-      </c>
+        <v>445</v>
+      </c>
+      <c r="X13" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="S14" t="s">
-        <v>394</v>
-      </c>
-      <c r="T14" t="s">
-        <v>395</v>
-      </c>
-      <c r="U14">
-        <v>10</v>
-      </c>
-      <c r="V14" t="s">
-        <v>103</v>
+        <v>441</v>
       </c>
       <c r="W14" t="s">
-        <v>81</v>
-      </c>
-      <c r="X14" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+        <v>447</v>
+      </c>
+      <c r="X14" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="W15" t="s">
-        <v>335</v>
-      </c>
-      <c r="X15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
+        <v>449</v>
+      </c>
+      <c r="X15" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="R16" t="s">
+        <v>451</v>
+      </c>
+      <c r="S16" t="s">
+        <v>452</v>
+      </c>
+      <c r="T16" t="s">
+        <v>453</v>
+      </c>
+      <c r="U16" t="s">
+        <v>422</v>
+      </c>
+      <c r="V16" t="s">
+        <v>454</v>
+      </c>
       <c r="W16" t="s">
-        <v>345</v>
-      </c>
-      <c r="X16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="23:24" x14ac:dyDescent="0.3">
+        <v>455</v>
+      </c>
+      <c r="X16" t="s">
+        <v>456</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>457</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="17" spans="23:27" x14ac:dyDescent="0.3">
       <c r="W17" t="s">
-        <v>355</v>
-      </c>
-      <c r="X17" t="b">
-        <v>0</v>
+        <v>459</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>437</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="18" spans="23:27" x14ac:dyDescent="0.3">
+      <c r="Y18" t="s">
+        <v>460</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>461</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="19" spans="23:27" x14ac:dyDescent="0.3">
+      <c r="Y19" t="s">
+        <v>462</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>463</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="20" spans="23:27" x14ac:dyDescent="0.3">
+      <c r="Y20" t="s">
+        <v>464</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>465</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>423</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Implement kanji progress tracking with Kafka integration and event handling
</commit_message>
<xml_diff>
--- a/repo-learning-path/test-data/learning-path-import-full-test.xlsx
+++ b/repo-learning-path/test-data/learning-path-import-full-test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DO_AN\BE_LMS\repo-learning-path\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F4D170E-4979-4DAE-85C0-1F0C307A22D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B06A4B6-58EF-4884-AA41-A02F65785E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="462">
   <si>
     <t>PackageName</t>
   </si>
@@ -1252,18 +1252,6 @@
   </si>
   <si>
     <t>Bo cau hoi tong hop cho ngu am, tu vung va ngu phap</t>
-  </si>
-  <si>
-    <t>Tieng Trung Nhap Mon</t>
-  </si>
-  <si>
-    <t>Hoc phat am pinyin va tu vung HSK 1</t>
-  </si>
-  <si>
-    <t>Tiet 1</t>
-  </si>
-  <si>
-    <t>On tap thanh mau va van mau</t>
   </si>
   <si>
     <t>Thu muc Tu vung va Ngu am</t>
@@ -3659,37 +3647,31 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:AB20"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="16.88671875" customWidth="1"/>
-    <col min="14" max="14" width="32.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="28.88671875" customWidth="1"/>
-    <col min="21" max="21" width="26.44140625" customWidth="1"/>
-    <col min="22" max="22" width="10.44140625" customWidth="1"/>
-    <col min="23" max="23" width="18.88671875" customWidth="1"/>
-    <col min="24" max="24" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="28" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="16.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="28.88671875" customWidth="1"/>
+    <col min="15" max="15" width="26.44140625" customWidth="1"/>
+    <col min="16" max="16" width="10.44140625" customWidth="1"/>
+    <col min="17" max="17" width="18.88671875" customWidth="1"/>
+    <col min="18" max="18" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="22" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3697,83 +3679,65 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>30</v>
+        <v>88</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>31</v>
+        <v>89</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>2</v>
+        <v>90</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>3</v>
+        <v>91</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>4</v>
+        <v>92</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>5</v>
+        <v>93</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="AA1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AB1" s="1"/>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="V1" s="1"/>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>407</v>
       </c>
@@ -3784,22 +3748,19 @@
         <v>409</v>
       </c>
       <c r="D2" t="s">
-        <v>147</v>
+        <v>410</v>
       </c>
       <c r="E2" t="s">
-        <v>410</v>
-      </c>
-      <c r="F2" t="s">
         <v>411</v>
       </c>
       <c r="G2" t="s">
-        <v>48</v>
+        <v>412</v>
       </c>
       <c r="H2" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="I2" t="s">
-        <v>413</v>
+        <v>105</v>
       </c>
       <c r="J2" t="s">
         <v>414</v>
@@ -3807,6 +3768,9 @@
       <c r="K2" t="s">
         <v>415</v>
       </c>
+      <c r="L2" t="s">
+        <v>104</v>
+      </c>
       <c r="M2" t="s">
         <v>416</v>
       </c>
@@ -3814,268 +3778,250 @@
         <v>417</v>
       </c>
       <c r="O2" t="s">
+        <v>418</v>
+      </c>
+      <c r="P2" t="s">
         <v>105</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
+        <v>50</v>
+      </c>
+      <c r="R2" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="Q3" t="s">
+        <v>420</v>
+      </c>
+      <c r="R3" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="Q4" t="s">
+        <v>136</v>
+      </c>
+      <c r="R4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="Q5" t="s">
+        <v>422</v>
+      </c>
+      <c r="R5" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="L6" t="s">
+        <v>104</v>
+      </c>
+      <c r="M6" t="s">
+        <v>423</v>
+      </c>
+      <c r="N6" t="s">
+        <v>424</v>
+      </c>
+      <c r="O6" t="s">
         <v>418</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="P6" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>352</v>
+      </c>
+      <c r="R6" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="Q7" t="s">
+        <v>425</v>
+      </c>
+      <c r="R7" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="Q8" t="s">
+        <v>426</v>
+      </c>
+      <c r="R8" t="s">
         <v>419</v>
       </c>
-      <c r="R2" t="s">
-        <v>104</v>
-      </c>
-      <c r="S2" t="s">
-        <v>420</v>
-      </c>
-      <c r="T2" t="s">
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="Q9" t="s">
+        <v>427</v>
+      </c>
+      <c r="R9" t="s">
         <v>421</v>
       </c>
-      <c r="U2" t="s">
-        <v>422</v>
-      </c>
-      <c r="V2" t="s">
-        <v>105</v>
-      </c>
-      <c r="W2" t="s">
-        <v>50</v>
-      </c>
-      <c r="X2" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="W3" t="s">
-        <v>424</v>
-      </c>
-      <c r="X3" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="W4" t="s">
-        <v>136</v>
-      </c>
-      <c r="X4" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="W5" t="s">
-        <v>426</v>
-      </c>
-      <c r="X5" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="R6" t="s">
-        <v>104</v>
-      </c>
-      <c r="S6" t="s">
-        <v>427</v>
-      </c>
-      <c r="T6" t="s">
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="L10" t="s">
         <v>428</v>
       </c>
-      <c r="U6" t="s">
-        <v>422</v>
-      </c>
-      <c r="V6" t="s">
-        <v>105</v>
-      </c>
-      <c r="W6" t="s">
-        <v>352</v>
-      </c>
-      <c r="X6" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="W7" t="s">
+      <c r="M10" t="s">
         <v>429</v>
       </c>
-      <c r="X7" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="W8" t="s">
+      <c r="N10" t="s">
         <v>430</v>
       </c>
-      <c r="X8" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="W9" t="s">
+      <c r="O10" t="s">
+        <v>418</v>
+      </c>
+      <c r="P10" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q10" t="s">
         <v>431</v>
       </c>
-      <c r="X9" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="R10" t="s">
         <v>432</v>
       </c>
-      <c r="S10" t="s">
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="Q11" t="s">
         <v>433</v>
       </c>
-      <c r="T10" t="s">
+      <c r="R11" t="s">
         <v>434</v>
       </c>
-      <c r="U10" t="s">
-        <v>422</v>
-      </c>
-      <c r="V10" t="s">
+      <c r="S11" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="L12" t="s">
+        <v>436</v>
+      </c>
+      <c r="M12" t="s">
+        <v>437</v>
+      </c>
+      <c r="N12" t="s">
+        <v>438</v>
+      </c>
+      <c r="O12" t="s">
+        <v>418</v>
+      </c>
+      <c r="P12" t="s">
         <v>103</v>
       </c>
-      <c r="W10" t="s">
-        <v>435</v>
-      </c>
-      <c r="X10" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="W11" t="s">
-        <v>437</v>
-      </c>
-      <c r="X11" t="s">
-        <v>438</v>
-      </c>
-      <c r="Y11" t="s">
+      <c r="Q12" t="s">
         <v>439</v>
       </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="R12" t="s">
         <v>440</v>
       </c>
-      <c r="S12" t="s">
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="Q13" t="s">
         <v>441</v>
       </c>
-      <c r="T12" t="s">
+      <c r="R13" t="s">
         <v>442</v>
       </c>
-      <c r="U12" t="s">
-        <v>422</v>
-      </c>
-      <c r="V12" t="s">
-        <v>103</v>
-      </c>
-      <c r="W12" t="s">
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="M14" t="s">
+        <v>437</v>
+      </c>
+      <c r="Q14" t="s">
         <v>443</v>
       </c>
-      <c r="X12" t="s">
+      <c r="R14" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="W13" t="s">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="Q15" t="s">
         <v>445</v>
       </c>
-      <c r="X13" t="s">
+      <c r="R15" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="S14" t="s">
-        <v>441</v>
-      </c>
-      <c r="W14" t="s">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="L16" t="s">
         <v>447</v>
       </c>
-      <c r="X14" t="s">
+      <c r="M16" t="s">
         <v>448</v>
       </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="W15" t="s">
+      <c r="N16" t="s">
         <v>449</v>
       </c>
-      <c r="X15" t="s">
+      <c r="O16" t="s">
+        <v>418</v>
+      </c>
+      <c r="P16" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="Q16" t="s">
+        <v>451</v>
+      </c>
       <c r="R16" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="S16" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="T16" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="U16" t="s">
-        <v>422</v>
-      </c>
-      <c r="V16" t="s">
-        <v>454</v>
-      </c>
-      <c r="W16" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="17" spans="17:21" x14ac:dyDescent="0.3">
+      <c r="Q17" t="s">
         <v>455</v>
       </c>
-      <c r="X16" t="s">
+      <c r="S17" t="s">
+        <v>433</v>
+      </c>
+      <c r="T17" t="s">
+        <v>48</v>
+      </c>
+      <c r="U17" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="18" spans="17:21" x14ac:dyDescent="0.3">
+      <c r="S18" t="s">
         <v>456</v>
       </c>
-      <c r="Y16" t="s">
+      <c r="T18" t="s">
         <v>457</v>
       </c>
-      <c r="Z16" t="s">
+      <c r="U18" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="19" spans="17:21" x14ac:dyDescent="0.3">
+      <c r="S19" t="s">
         <v>458</v>
       </c>
-      <c r="AA16" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="17" spans="23:27" x14ac:dyDescent="0.3">
-      <c r="W17" t="s">
+      <c r="T19" t="s">
         <v>459</v>
       </c>
-      <c r="Y17" t="s">
-        <v>437</v>
-      </c>
-      <c r="Z17" t="s">
-        <v>48</v>
-      </c>
-      <c r="AA17" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="18" spans="23:27" x14ac:dyDescent="0.3">
-      <c r="Y18" t="s">
+      <c r="U19" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="20" spans="17:21" x14ac:dyDescent="0.3">
+      <c r="S20" t="s">
         <v>460</v>
       </c>
-      <c r="Z18" t="s">
+      <c r="T20" t="s">
         <v>461</v>
       </c>
-      <c r="AA18" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="19" spans="23:27" x14ac:dyDescent="0.3">
-      <c r="Y19" t="s">
-        <v>462</v>
-      </c>
-      <c r="Z19" t="s">
-        <v>463</v>
-      </c>
-      <c r="AA19" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="20" spans="23:27" x14ac:dyDescent="0.3">
-      <c r="Y20" t="s">
-        <v>464</v>
-      </c>
-      <c r="Z20" t="s">
-        <v>465</v>
-      </c>
-      <c r="AA20" t="s">
-        <v>423</v>
+      <c r="U20" t="s">
+        <v>419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Enhance hierarchical import services with customizable required headers
</commit_message>
<xml_diff>
--- a/repo-learning-path/test-data/learning-path-import-full-test.xlsx
+++ b/repo-learning-path/test-data/learning-path-import-full-test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DO_AN\BE_LMS\repo-learning-path\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B06A4B6-58EF-4884-AA41-A02F65785E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F2A1729-FB87-409A-A342-C59A0563F726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="438">
   <si>
     <t>PackageName</t>
   </si>
@@ -105,24 +105,6 @@
     <t>QuizSheet</t>
   </si>
   <si>
-    <t>SubjectName</t>
-  </si>
-  <si>
-    <t>SubjectCode</t>
-  </si>
-  <si>
-    <t>SubjectDescription</t>
-  </si>
-  <si>
-    <t>SlotName</t>
-  </si>
-  <si>
-    <t>SlotNumber</t>
-  </si>
-  <si>
-    <t>SlotDescription</t>
-  </si>
-  <si>
     <t>Term</t>
   </si>
   <si>
@@ -165,18 +147,9 @@
     <t>CharactersJson</t>
   </si>
   <si>
-    <t>Flashcard subject desc</t>
-  </si>
-  <si>
-    <t>FC Slot</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
-    <t>Flashcard slot desc</t>
-  </si>
-  <si>
     <t>你好</t>
   </si>
   <si>
@@ -231,9 +204,6 @@
     <t>OriginTextCn</t>
   </si>
   <si>
-    <t>OriginTextEn</t>
-  </si>
-  <si>
     <t>StrokeAnimationUrl</t>
   </si>
   <si>
@@ -267,9 +237,6 @@
     <t>https://example.com/stroke/ri.gif</t>
   </si>
   <si>
-    <t>PR101</t>
-  </si>
-  <si>
     <t>b</t>
   </si>
   <si>
@@ -468,18 +435,6 @@
     <t>[{"char":"再"},{"char":"见"}]</t>
   </si>
   <si>
-    <t>CHN101</t>
-  </si>
-  <si>
-    <t>Tiếng Trung Cơ Bản</t>
-  </si>
-  <si>
-    <t>Tiếng Trung dành cho người mới bắt đầu</t>
-  </si>
-  <si>
-    <t>Từ vựng chào hỏi cơ bản</t>
-  </si>
-  <si>
     <t>Thư mục Giao Tiếp</t>
   </si>
   <si>
@@ -672,27 +627,9 @@
     <t xml:space="preserve">Các kí tự hán tự luyện theo bài học </t>
   </si>
   <si>
-    <t>Bài 1: Gia đình</t>
-  </si>
-  <si>
     <t>Tìm hiểu nguồn gốc các chữ Hán cơ bản qua hình ảnh</t>
   </si>
   <si>
-    <t>Hán Tự Nhập Môn</t>
-  </si>
-  <si>
-    <t>HAN101</t>
-  </si>
-  <si>
-    <t>Khóa học về cấu tạo và ý nghĩa chữ Hán</t>
-  </si>
-  <si>
-    <t>Tiết học Bộ Thủ</t>
-  </si>
-  <si>
-    <t>Phân tích các bộ thủ tượng hình</t>
-  </si>
-  <si>
     <t>Thư mục Nguồn Gốc</t>
   </si>
   <si>
@@ -996,18 +933,6 @@
     <t>Học cách phát âm tiếng Trung chuẩn xác</t>
   </si>
   <si>
-    <t>Ngữ Âm Cơ Bản</t>
-  </si>
-  <si>
-    <t>Khóa học về thanh mẫu, vận mẫu và thanh điệu</t>
-  </si>
-  <si>
-    <t>Tiết Học Ngữ Âm</t>
-  </si>
-  <si>
-    <t>Luyện tập các âm môi và đầu lưỡi</t>
-  </si>
-  <si>
     <t>Thư mục Ngữ Âm</t>
   </si>
   <si>
@@ -1411,6 +1336,9 @@
   </si>
   <si>
     <t>4</t>
+  </si>
+  <si>
+    <t>OriginTextVi</t>
   </si>
 </sst>
 </file>
@@ -1838,40 +1766,40 @@
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>376</v>
+        <v>351</v>
       </c>
       <c r="B2" t="s">
-        <v>377</v>
+        <v>352</v>
       </c>
       <c r="C2" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="D2" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="E2" t="s">
-        <v>380</v>
+        <v>355</v>
       </c>
       <c r="F2" t="s">
-        <v>381</v>
+        <v>356</v>
       </c>
       <c r="G2" t="s">
-        <v>382</v>
+        <v>357</v>
       </c>
       <c r="H2" t="s">
-        <v>383</v>
+        <v>358</v>
       </c>
       <c r="I2" t="s">
-        <v>384</v>
+        <v>359</v>
       </c>
       <c r="J2" t="s">
-        <v>385</v>
+        <v>360</v>
       </c>
       <c r="K2">
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>386</v>
+        <v>361</v>
       </c>
       <c r="M2" t="s">
         <v>16</v>
@@ -1888,16 +1816,16 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="I3" t="s">
-        <v>387</v>
+        <v>362</v>
       </c>
       <c r="J3" t="s">
-        <v>388</v>
+        <v>363</v>
       </c>
       <c r="K3">
         <v>2</v>
       </c>
       <c r="L3" t="s">
-        <v>389</v>
+        <v>364</v>
       </c>
       <c r="M3" t="s">
         <v>18</v>
@@ -1914,16 +1842,16 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="I4" t="s">
-        <v>390</v>
+        <v>365</v>
       </c>
       <c r="J4" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="K4">
         <v>3</v>
       </c>
       <c r="L4" t="s">
-        <v>392</v>
+        <v>367</v>
       </c>
       <c r="M4" t="s">
         <v>20</v>
@@ -1940,34 +1868,34 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
-        <v>393</v>
+        <v>368</v>
       </c>
       <c r="D5" t="s">
-        <v>394</v>
+        <v>369</v>
       </c>
       <c r="E5" t="s">
-        <v>395</v>
+        <v>370</v>
       </c>
       <c r="F5" t="s">
-        <v>396</v>
+        <v>371</v>
       </c>
       <c r="G5" t="s">
-        <v>397</v>
+        <v>372</v>
       </c>
       <c r="H5" t="s">
-        <v>398</v>
+        <v>373</v>
       </c>
       <c r="I5" t="s">
-        <v>399</v>
+        <v>374</v>
       </c>
       <c r="J5" t="s">
-        <v>400</v>
+        <v>375</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
       <c r="L5" t="s">
-        <v>401</v>
+        <v>376</v>
       </c>
       <c r="M5" t="s">
         <v>22</v>
@@ -1984,16 +1912,16 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="I6" t="s">
-        <v>402</v>
+        <v>377</v>
       </c>
       <c r="J6" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="K6">
         <v>2</v>
       </c>
       <c r="L6" t="s">
-        <v>404</v>
+        <v>379</v>
       </c>
       <c r="M6" t="s">
         <v>24</v>
@@ -2016,35 +1944,29 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="38.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="22.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="39.88671875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="24.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="39.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="24.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2052,34 +1974,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>32</v>
@@ -2105,236 +2027,200 @@
       <c r="T1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="V1" s="1" t="s">
+      <c r="U1" s="1"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G2" t="s">
         <v>41</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="H2" t="s">
         <v>42</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="I2" t="s">
         <v>43</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="J2" t="s">
         <v>44</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="K2" t="s">
         <v>45</v>
       </c>
-      <c r="AA1" s="1"/>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="L2" t="s">
+        <v>46</v>
+      </c>
+      <c r="M2" t="s">
+        <v>47</v>
+      </c>
+      <c r="N2" t="s">
+        <v>48</v>
+      </c>
+      <c r="O2" t="s">
+        <v>49</v>
+      </c>
+      <c r="P2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>51</v>
+      </c>
+      <c r="R2" t="s">
+        <v>52</v>
+      </c>
+      <c r="S2" t="s">
+        <v>53</v>
+      </c>
+      <c r="T2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H3" t="s">
+        <v>102</v>
+      </c>
+      <c r="I3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J3" t="s">
+        <v>104</v>
+      </c>
+      <c r="K3" t="s">
+        <v>105</v>
+      </c>
+      <c r="L3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" t="s">
         <v>106</v>
       </c>
-      <c r="B2" t="s">
+      <c r="N3" t="s">
+        <v>108</v>
+      </c>
+      <c r="O3" t="s">
         <v>107</v>
       </c>
-      <c r="C2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="P3" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>110</v>
+      </c>
+      <c r="R3" t="s">
+        <v>111</v>
+      </c>
+      <c r="S3" t="s">
+        <v>112</v>
+      </c>
+      <c r="T3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>114</v>
+      </c>
+      <c r="H4" t="s">
+        <v>115</v>
+      </c>
+      <c r="I4" t="s">
+        <v>116</v>
+      </c>
+      <c r="J4" t="s">
+        <v>117</v>
+      </c>
+      <c r="K4" t="s">
+        <v>105</v>
+      </c>
+      <c r="L4" t="s">
         <v>46</v>
       </c>
-      <c r="F2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H2" t="s">
-        <v>49</v>
-      </c>
-      <c r="I2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J2" t="s">
-        <v>110</v>
-      </c>
-      <c r="K2" t="s">
-        <v>111</v>
-      </c>
-      <c r="L2" t="s">
-        <v>108</v>
-      </c>
-      <c r="M2" t="s">
-        <v>50</v>
-      </c>
-      <c r="N2" t="s">
-        <v>51</v>
-      </c>
-      <c r="O2" t="s">
-        <v>52</v>
-      </c>
-      <c r="P2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>54</v>
-      </c>
-      <c r="R2" t="s">
-        <v>55</v>
-      </c>
-      <c r="S2" t="s">
-        <v>56</v>
-      </c>
-      <c r="T2" t="s">
-        <v>57</v>
-      </c>
-      <c r="U2" t="s">
-        <v>58</v>
-      </c>
-      <c r="V2" t="s">
-        <v>59</v>
-      </c>
-      <c r="W2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X2" t="s">
-        <v>61</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M3" t="s">
-        <v>112</v>
-      </c>
-      <c r="N3" t="s">
+      <c r="M4" t="s">
+        <v>118</v>
+      </c>
+      <c r="N4" t="s">
+        <v>119</v>
+      </c>
+      <c r="O4" t="s">
+        <v>120</v>
+      </c>
+      <c r="P4" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>122</v>
+      </c>
+      <c r="R4" t="s">
+        <v>123</v>
+      </c>
+      <c r="S4" t="s">
+        <v>124</v>
+      </c>
+      <c r="T4" t="s">
         <v>113</v>
       </c>
-      <c r="O3" t="s">
-        <v>114</v>
-      </c>
-      <c r="P3" t="s">
-        <v>115</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>116</v>
-      </c>
-      <c r="R3" t="s">
-        <v>55</v>
-      </c>
-      <c r="S3" t="s">
-        <v>117</v>
-      </c>
-      <c r="T3" t="s">
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>125</v>
+      </c>
+      <c r="H5" t="s">
+        <v>126</v>
+      </c>
+      <c r="I5" t="s">
+        <v>127</v>
+      </c>
+      <c r="J5" t="s">
+        <v>128</v>
+      </c>
+      <c r="K5" t="s">
+        <v>105</v>
+      </c>
+      <c r="L5" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" t="s">
+        <v>129</v>
+      </c>
+      <c r="N5" t="s">
         <v>119</v>
       </c>
-      <c r="U3" t="s">
-        <v>118</v>
-      </c>
-      <c r="V3" t="s">
-        <v>120</v>
-      </c>
-      <c r="W3" t="s">
-        <v>121</v>
-      </c>
-      <c r="X3" t="s">
-        <v>122</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M4" t="s">
-        <v>125</v>
-      </c>
-      <c r="N4" t="s">
-        <v>126</v>
-      </c>
-      <c r="O4" t="s">
-        <v>127</v>
-      </c>
-      <c r="P4" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>116</v>
-      </c>
-      <c r="R4" t="s">
-        <v>55</v>
-      </c>
-      <c r="S4" t="s">
-        <v>129</v>
-      </c>
-      <c r="T4" t="s">
+      <c r="O5" t="s">
         <v>130</v>
       </c>
-      <c r="U4" t="s">
+      <c r="P5" t="s">
         <v>131</v>
       </c>
-      <c r="V4" t="s">
+      <c r="Q5" t="s">
         <v>132</v>
       </c>
-      <c r="W4" t="s">
+      <c r="R5" t="s">
         <v>133</v>
       </c>
-      <c r="X4" t="s">
+      <c r="S5" t="s">
         <v>134</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="T5" t="s">
         <v>135</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M5" t="s">
-        <v>136</v>
-      </c>
-      <c r="N5" t="s">
-        <v>137</v>
-      </c>
-      <c r="O5" t="s">
-        <v>138</v>
-      </c>
-      <c r="P5" t="s">
-        <v>139</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>116</v>
-      </c>
-      <c r="R5" t="s">
-        <v>55</v>
-      </c>
-      <c r="S5" t="s">
-        <v>140</v>
-      </c>
-      <c r="T5" t="s">
-        <v>130</v>
-      </c>
-      <c r="U5" t="s">
-        <v>141</v>
-      </c>
-      <c r="V5" t="s">
-        <v>142</v>
-      </c>
-      <c r="W5" t="s">
-        <v>143</v>
-      </c>
-      <c r="X5" t="s">
-        <v>144</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -2344,38 +2230,32 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="22.88671875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="33.33203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="24.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="33.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="24.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2383,34 +2263,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>32</v>
@@ -2436,280 +2316,244 @@
       <c r="T1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z1" s="1" t="s">
+      <c r="U1" s="1"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H2" t="s">
+        <v>141</v>
+      </c>
+      <c r="I2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J2" t="s">
+        <v>143</v>
+      </c>
+      <c r="K2" t="s">
         <v>45</v>
       </c>
-      <c r="AA1" s="1"/>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="L2" t="s">
+        <v>46</v>
+      </c>
+      <c r="M2" t="s">
+        <v>144</v>
+      </c>
+      <c r="N2" t="s">
+        <v>145</v>
+      </c>
+      <c r="O2" t="s">
+        <v>146</v>
+      </c>
+      <c r="P2" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q2" t="s">
         <v>148</v>
       </c>
-      <c r="D2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="R2" t="s">
         <v>149</v>
       </c>
-      <c r="F2" t="s">
-        <v>215</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="S2" t="s">
         <v>150</v>
       </c>
-      <c r="I2" t="s">
+      <c r="T2" t="s">
         <v>151</v>
       </c>
-      <c r="J2" t="s">
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
         <v>152</v>
       </c>
-      <c r="K2" t="s">
+      <c r="H3" t="s">
         <v>153</v>
       </c>
-      <c r="L2" t="s">
+      <c r="I3" t="s">
         <v>154</v>
       </c>
-      <c r="M2" t="s">
+      <c r="J3" t="s">
+        <v>154</v>
+      </c>
+      <c r="K3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" t="s">
         <v>155</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N3" t="s">
         <v>156</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O3" t="s">
         <v>157</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P3" t="s">
         <v>158</v>
       </c>
-      <c r="Q2" t="s">
-        <v>54</v>
-      </c>
-      <c r="R2" t="s">
+      <c r="Q3" t="s">
+        <v>159</v>
+      </c>
+      <c r="R3" t="s">
+        <v>160</v>
+      </c>
+      <c r="S3" t="s">
+        <v>161</v>
+      </c>
+      <c r="T3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>163</v>
+      </c>
+      <c r="H4" t="s">
+        <v>164</v>
+      </c>
+      <c r="I4" t="s">
+        <v>165</v>
+      </c>
+      <c r="J4" t="s">
+        <v>166</v>
+      </c>
+      <c r="K4" t="s">
+        <v>45</v>
+      </c>
+      <c r="L4" t="s">
+        <v>46</v>
+      </c>
+      <c r="M4" t="s">
+        <v>167</v>
+      </c>
+      <c r="N4" t="s">
+        <v>168</v>
+      </c>
+      <c r="O4" t="s">
+        <v>169</v>
+      </c>
+      <c r="P4" t="s">
+        <v>170</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>171</v>
+      </c>
+      <c r="R4" t="s">
+        <v>172</v>
+      </c>
+      <c r="S4" t="s">
+        <v>173</v>
+      </c>
+      <c r="T4" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>175</v>
+      </c>
+      <c r="H5" t="s">
+        <v>176</v>
+      </c>
+      <c r="I5" t="s">
+        <v>177</v>
+      </c>
+      <c r="J5" t="s">
+        <v>178</v>
+      </c>
+      <c r="K5" t="s">
+        <v>105</v>
+      </c>
+      <c r="L5" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" t="s">
+        <v>179</v>
+      </c>
+      <c r="N5" t="s">
+        <v>180</v>
+      </c>
+      <c r="O5" t="s">
+        <v>181</v>
+      </c>
+      <c r="P5" t="s">
+        <v>182</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>183</v>
+      </c>
+      <c r="R5" t="s">
+        <v>184</v>
+      </c>
+      <c r="S5" t="s">
+        <v>185</v>
+      </c>
+      <c r="T5" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>187</v>
+      </c>
+      <c r="H6" t="s">
+        <v>188</v>
+      </c>
+      <c r="I6" t="s">
+        <v>189</v>
+      </c>
+      <c r="J6" t="s">
+        <v>190</v>
+      </c>
+      <c r="K6" t="s">
         <v>55</v>
       </c>
-      <c r="S2" t="s">
-        <v>159</v>
-      </c>
-      <c r="T2" t="s">
-        <v>160</v>
-      </c>
-      <c r="U2" t="s">
-        <v>161</v>
-      </c>
-      <c r="V2" t="s">
-        <v>162</v>
-      </c>
-      <c r="W2" t="s">
-        <v>163</v>
-      </c>
-      <c r="X2" t="s">
-        <v>164</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>165</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M3" t="s">
-        <v>167</v>
-      </c>
-      <c r="N3" t="s">
-        <v>168</v>
-      </c>
-      <c r="O3" t="s">
-        <v>169</v>
-      </c>
-      <c r="P3" t="s">
-        <v>169</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>54</v>
-      </c>
-      <c r="R3" t="s">
-        <v>55</v>
-      </c>
-      <c r="S3" t="s">
-        <v>170</v>
-      </c>
-      <c r="T3" t="s">
-        <v>171</v>
-      </c>
-      <c r="U3" t="s">
-        <v>172</v>
-      </c>
-      <c r="V3" t="s">
-        <v>173</v>
-      </c>
-      <c r="W3" t="s">
-        <v>174</v>
-      </c>
-      <c r="X3" t="s">
-        <v>175</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M4" t="s">
-        <v>178</v>
-      </c>
-      <c r="N4" t="s">
-        <v>179</v>
-      </c>
-      <c r="O4" t="s">
-        <v>180</v>
-      </c>
-      <c r="P4" t="s">
-        <v>181</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>54</v>
-      </c>
-      <c r="R4" t="s">
-        <v>55</v>
-      </c>
-      <c r="S4" t="s">
-        <v>182</v>
-      </c>
-      <c r="T4" t="s">
-        <v>183</v>
-      </c>
-      <c r="U4" t="s">
-        <v>184</v>
-      </c>
-      <c r="V4" t="s">
-        <v>185</v>
-      </c>
-      <c r="W4" t="s">
-        <v>186</v>
-      </c>
-      <c r="X4" t="s">
-        <v>187</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>188</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M5" t="s">
-        <v>190</v>
-      </c>
-      <c r="N5" t="s">
+      <c r="L6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M6" t="s">
         <v>191</v>
       </c>
-      <c r="O5" t="s">
+      <c r="N6" t="s">
         <v>192</v>
       </c>
-      <c r="P5" t="s">
+      <c r="O6" t="s">
         <v>193</v>
       </c>
-      <c r="Q5" t="s">
-        <v>116</v>
-      </c>
-      <c r="R5" t="s">
-        <v>55</v>
-      </c>
-      <c r="S5" t="s">
+      <c r="P6" t="s">
         <v>194</v>
       </c>
-      <c r="T5" t="s">
+      <c r="Q6" t="s">
         <v>195</v>
       </c>
-      <c r="U5" t="s">
+      <c r="R6" t="s">
         <v>196</v>
       </c>
-      <c r="V5" t="s">
+      <c r="S6" t="s">
         <v>197</v>
       </c>
-      <c r="W5" t="s">
-        <v>198</v>
-      </c>
-      <c r="X5" t="s">
-        <v>199</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>200</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M6" t="s">
-        <v>202</v>
-      </c>
-      <c r="N6" t="s">
-        <v>203</v>
-      </c>
-      <c r="O6" t="s">
-        <v>204</v>
-      </c>
-      <c r="P6" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>64</v>
-      </c>
-      <c r="R6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S6" t="s">
-        <v>206</v>
-      </c>
       <c r="T6" t="s">
-        <v>207</v>
-      </c>
-      <c r="U6" t="s">
-        <v>208</v>
-      </c>
-      <c r="V6" t="s">
-        <v>209</v>
-      </c>
-      <c r="W6" t="s">
-        <v>210</v>
-      </c>
-      <c r="X6" t="s">
-        <v>211</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>212</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>406</v>
+        <v>381</v>
       </c>
     </row>
   </sheetData>
@@ -2719,48 +2563,42 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:AK6"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="16.88671875" customWidth="1"/>
-    <col min="28" max="28" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="30.77734375" customWidth="1"/>
-    <col min="31" max="31" width="29" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="28" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="15" customWidth="1"/>
-    <col min="36" max="36" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.88671875" customWidth="1"/>
+    <col min="22" max="22" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="30.77734375" customWidth="1"/>
+    <col min="25" max="25" width="29" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="28" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="15" customWidth="1"/>
+    <col min="30" max="30" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2768,34 +2606,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>32</v>
@@ -2822,447 +2660,411 @@
         <v>39</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>43</v>
+        <v>437</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="AA1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="AE1" s="1"/>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E2" t="s">
+        <v>203</v>
+      </c>
+      <c r="F2" t="s">
+        <v>204</v>
+      </c>
+      <c r="G2" t="s">
         <v>65</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="H2" t="s">
+        <v>205</v>
+      </c>
+      <c r="I2" t="s">
+        <v>206</v>
+      </c>
+      <c r="J2" t="s">
+        <v>207</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
+        <v>46</v>
+      </c>
+      <c r="M2" t="s">
+        <v>208</v>
+      </c>
+      <c r="N2" t="s">
+        <v>209</v>
+      </c>
+      <c r="O2" t="s">
+        <v>210</v>
+      </c>
+      <c r="P2" t="s">
         <v>66</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="Q2" t="s">
+        <v>211</v>
+      </c>
+      <c r="R2" t="s">
+        <v>212</v>
+      </c>
+      <c r="S2" t="s">
+        <v>213</v>
+      </c>
+      <c r="T2" t="s">
         <v>67</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="U2" t="s">
+        <v>214</v>
+      </c>
+      <c r="V2" t="s">
+        <v>215</v>
+      </c>
+      <c r="W2" t="s">
+        <v>216</v>
+      </c>
+      <c r="X2" t="s">
         <v>68</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="Y2" t="s">
         <v>69</v>
       </c>
-      <c r="AF1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK1" s="1"/>
-    </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>321</v>
-      </c>
-      <c r="B2" t="s">
-        <v>216</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="Z2" t="s">
+        <v>213</v>
+      </c>
+      <c r="AA2" t="s">
         <v>217</v>
       </c>
-      <c r="D2" t="s">
+      <c r="AB2" t="s">
         <v>218</v>
       </c>
-      <c r="E2" t="s">
+      <c r="AC2" t="s">
         <v>219</v>
       </c>
-      <c r="F2" t="s">
+      <c r="AD2" t="s">
         <v>220</v>
       </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2" t="s">
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
         <v>221</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H3" t="s">
         <v>222</v>
       </c>
-      <c r="J2" t="s">
+      <c r="I3" t="s">
         <v>223</v>
       </c>
-      <c r="K2" t="s">
+      <c r="J3" t="s">
         <v>224</v>
       </c>
-      <c r="L2" t="s">
+      <c r="K3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" t="s">
         <v>225</v>
       </c>
-      <c r="M2" t="s">
-        <v>75</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="N3" t="s">
         <v>226</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O3" t="s">
         <v>227</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P3" t="s">
         <v>228</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q3" t="s">
+        <v>229</v>
+      </c>
+      <c r="R3" t="s">
+        <v>230</v>
+      </c>
+      <c r="S3" t="s">
+        <v>231</v>
+      </c>
+      <c r="T3" t="s">
+        <v>232</v>
+      </c>
+      <c r="W3" t="s">
+        <v>233</v>
+      </c>
+      <c r="X3" t="s">
+        <v>234</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>235</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>231</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>236</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>237</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>238</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>240</v>
+      </c>
+      <c r="H4" t="s">
+        <v>241</v>
+      </c>
+      <c r="I4" t="s">
+        <v>242</v>
+      </c>
+      <c r="J4" t="s">
+        <v>243</v>
+      </c>
+      <c r="K4" t="s">
         <v>20</v>
       </c>
-      <c r="R2" t="s">
-        <v>55</v>
-      </c>
-      <c r="S2" t="s">
-        <v>229</v>
-      </c>
-      <c r="T2" t="s">
-        <v>230</v>
-      </c>
-      <c r="U2" t="s">
-        <v>231</v>
-      </c>
-      <c r="V2" t="s">
-        <v>76</v>
-      </c>
-      <c r="W2" t="s">
-        <v>232</v>
-      </c>
-      <c r="X2" t="s">
-        <v>233</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>234</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>77</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>235</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>236</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>237</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>78</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>79</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>234</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>238</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>239</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>240</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="M3" t="s">
-        <v>242</v>
-      </c>
-      <c r="N3" t="s">
-        <v>243</v>
-      </c>
-      <c r="O3" t="s">
+      <c r="L4" t="s">
+        <v>46</v>
+      </c>
+      <c r="M4" t="s">
         <v>244</v>
       </c>
-      <c r="P3" t="s">
+      <c r="N4" t="s">
         <v>245</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="O4" t="s">
+        <v>246</v>
+      </c>
+      <c r="P4" t="s">
+        <v>247</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>248</v>
+      </c>
+      <c r="R4" t="s">
+        <v>249</v>
+      </c>
+      <c r="S4" t="s">
+        <v>250</v>
+      </c>
+      <c r="T4" t="s">
+        <v>251</v>
+      </c>
+      <c r="U4" t="s">
+        <v>252</v>
+      </c>
+      <c r="V4" t="s">
+        <v>253</v>
+      </c>
+      <c r="W4" t="s">
+        <v>254</v>
+      </c>
+      <c r="X4" t="s">
+        <v>255</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>256</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>258</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>259</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>260</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>262</v>
+      </c>
+      <c r="H5" t="s">
+        <v>263</v>
+      </c>
+      <c r="I5" t="s">
+        <v>264</v>
+      </c>
+      <c r="J5" t="s">
+        <v>265</v>
+      </c>
+      <c r="K5" t="s">
         <v>20</v>
       </c>
-      <c r="R3" t="s">
-        <v>55</v>
-      </c>
-      <c r="S3" t="s">
-        <v>246</v>
-      </c>
-      <c r="T3" t="s">
-        <v>247</v>
-      </c>
-      <c r="U3" t="s">
-        <v>248</v>
-      </c>
-      <c r="V3" t="s">
-        <v>249</v>
-      </c>
-      <c r="W3" t="s">
-        <v>250</v>
-      </c>
-      <c r="X3" t="s">
-        <v>251</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>252</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>253</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>254</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>255</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>256</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>252</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>257</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>258</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>259</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="M4" t="s">
-        <v>261</v>
-      </c>
-      <c r="N4" t="s">
-        <v>262</v>
-      </c>
-      <c r="O4" t="s">
-        <v>263</v>
-      </c>
-      <c r="P4" t="s">
-        <v>264</v>
-      </c>
-      <c r="Q4" t="s">
+      <c r="L5" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" t="s">
+        <v>266</v>
+      </c>
+      <c r="N5" t="s">
+        <v>267</v>
+      </c>
+      <c r="O5" t="s">
+        <v>268</v>
+      </c>
+      <c r="P5" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>175</v>
+      </c>
+      <c r="R5" t="s">
+        <v>270</v>
+      </c>
+      <c r="S5" t="s">
+        <v>271</v>
+      </c>
+      <c r="T5" t="s">
+        <v>272</v>
+      </c>
+      <c r="W5" t="s">
+        <v>273</v>
+      </c>
+      <c r="X5" t="s">
+        <v>274</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>275</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>185</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>276</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>277</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>280</v>
+      </c>
+      <c r="H6" t="s">
+        <v>281</v>
+      </c>
+      <c r="I6" t="s">
+        <v>282</v>
+      </c>
+      <c r="J6" t="s">
+        <v>283</v>
+      </c>
+      <c r="K6" t="s">
         <v>20</v>
       </c>
-      <c r="R4" t="s">
-        <v>55</v>
-      </c>
-      <c r="S4" t="s">
-        <v>265</v>
-      </c>
-      <c r="T4" t="s">
-        <v>266</v>
-      </c>
-      <c r="U4" t="s">
-        <v>267</v>
-      </c>
-      <c r="V4" t="s">
-        <v>268</v>
-      </c>
-      <c r="W4" t="s">
-        <v>269</v>
-      </c>
-      <c r="X4" t="s">
-        <v>270</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>271</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>272</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>273</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>274</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>275</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>276</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>277</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>278</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>279</v>
-      </c>
-      <c r="AH4" t="s">
+      <c r="L6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M6" t="s">
+        <v>284</v>
+      </c>
+      <c r="N6" t="s">
+        <v>285</v>
+      </c>
+      <c r="O6" t="s">
+        <v>286</v>
+      </c>
+      <c r="P6" t="s">
+        <v>287</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>288</v>
+      </c>
+      <c r="R6" t="s">
+        <v>289</v>
+      </c>
+      <c r="S6" t="s">
+        <v>290</v>
+      </c>
+      <c r="T6" t="s">
+        <v>291</v>
+      </c>
+      <c r="U6" t="s">
+        <v>292</v>
+      </c>
+      <c r="V6" t="s">
+        <v>293</v>
+      </c>
+      <c r="W6" t="s">
+        <v>294</v>
+      </c>
+      <c r="X6" t="s">
+        <v>295</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>296</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>297</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>298</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>299</v>
+      </c>
+      <c r="AC6" t="s">
         <v>280</v>
       </c>
-      <c r="AI4" t="s">
-        <v>281</v>
-      </c>
-      <c r="AJ4" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="M5" t="s">
-        <v>283</v>
-      </c>
-      <c r="N5" t="s">
-        <v>284</v>
-      </c>
-      <c r="O5" t="s">
-        <v>285</v>
-      </c>
-      <c r="P5" t="s">
-        <v>286</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>20</v>
-      </c>
-      <c r="R5" t="s">
-        <v>55</v>
-      </c>
-      <c r="S5" t="s">
-        <v>287</v>
-      </c>
-      <c r="T5" t="s">
-        <v>288</v>
-      </c>
-      <c r="U5" t="s">
-        <v>289</v>
-      </c>
-      <c r="V5" t="s">
-        <v>290</v>
-      </c>
-      <c r="W5" t="s">
-        <v>190</v>
-      </c>
-      <c r="X5" t="s">
-        <v>291</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>292</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>293</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>294</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>295</v>
-      </c>
-      <c r="AE5" t="s">
-        <v>296</v>
-      </c>
-      <c r="AF5" t="s">
-        <v>200</v>
-      </c>
-      <c r="AG5" t="s">
-        <v>297</v>
-      </c>
-      <c r="AH5" t="s">
-        <v>298</v>
-      </c>
-      <c r="AI5" t="s">
-        <v>299</v>
-      </c>
-      <c r="AJ5" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.3">
-      <c r="M6" t="s">
-        <v>301</v>
-      </c>
-      <c r="N6" t="s">
-        <v>302</v>
-      </c>
-      <c r="O6" t="s">
-        <v>303</v>
-      </c>
-      <c r="P6" t="s">
-        <v>304</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>20</v>
-      </c>
-      <c r="R6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S6" t="s">
-        <v>305</v>
-      </c>
-      <c r="T6" t="s">
-        <v>306</v>
-      </c>
-      <c r="U6" t="s">
-        <v>307</v>
-      </c>
-      <c r="V6" t="s">
-        <v>308</v>
-      </c>
-      <c r="W6" t="s">
-        <v>309</v>
-      </c>
-      <c r="X6" t="s">
-        <v>310</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>311</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>312</v>
-      </c>
-      <c r="AA6" t="s">
-        <v>313</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>314</v>
-      </c>
-      <c r="AC6" t="s">
-        <v>315</v>
-      </c>
       <c r="AD6" t="s">
-        <v>316</v>
-      </c>
-      <c r="AE6" t="s">
-        <v>317</v>
-      </c>
-      <c r="AF6" t="s">
-        <v>318</v>
-      </c>
-      <c r="AG6" t="s">
-        <v>319</v>
-      </c>
-      <c r="AH6" t="s">
-        <v>320</v>
-      </c>
-      <c r="AI6" t="s">
-        <v>301</v>
-      </c>
-      <c r="AJ6" t="s">
-        <v>405</v>
+        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -3272,38 +3074,32 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="36.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="30" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="36.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="30" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3311,34 +3107,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>32</v>
@@ -3364,280 +3160,244 @@
       <c r="T1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AA1" s="1"/>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="U1" s="1"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>375</v>
+        <v>350</v>
       </c>
       <c r="B2" t="s">
+        <v>301</v>
+      </c>
+      <c r="C2" t="s">
+        <v>302</v>
+      </c>
+      <c r="D2" t="s">
+        <v>303</v>
+      </c>
+      <c r="E2" t="s">
+        <v>304</v>
+      </c>
+      <c r="F2" t="s">
+        <v>305</v>
+      </c>
+      <c r="G2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H2" t="s">
+        <v>306</v>
+      </c>
+      <c r="I2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J2" t="s">
+        <v>71</v>
+      </c>
+      <c r="K2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L2" t="s">
+        <v>46</v>
+      </c>
+      <c r="M2" t="s">
+        <v>73</v>
+      </c>
+      <c r="N2" t="s">
+        <v>307</v>
+      </c>
+      <c r="O2" t="s">
+        <v>74</v>
+      </c>
+      <c r="P2" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>308</v>
+      </c>
+      <c r="R2" t="s">
+        <v>308</v>
+      </c>
+      <c r="S2" t="s">
+        <v>309</v>
+      </c>
+      <c r="T2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>310</v>
+      </c>
+      <c r="H3" t="s">
+        <v>311</v>
+      </c>
+      <c r="I3" t="s">
+        <v>310</v>
+      </c>
+      <c r="J3" t="s">
+        <v>312</v>
+      </c>
+      <c r="K3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" t="s">
+        <v>313</v>
+      </c>
+      <c r="N3" t="s">
+        <v>314</v>
+      </c>
+      <c r="O3" t="s">
+        <v>315</v>
+      </c>
+      <c r="P3" t="s">
+        <v>316</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>317</v>
+      </c>
+      <c r="R3" t="s">
+        <v>317</v>
+      </c>
+      <c r="S3" t="s">
+        <v>318</v>
+      </c>
+      <c r="T3" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>320</v>
+      </c>
+      <c r="H4" t="s">
+        <v>321</v>
+      </c>
+      <c r="I4" t="s">
+        <v>320</v>
+      </c>
+      <c r="J4" t="s">
         <v>322</v>
       </c>
-      <c r="C2" t="s">
+      <c r="K4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L4" t="s">
+        <v>46</v>
+      </c>
+      <c r="M4" t="s">
         <v>323</v>
       </c>
-      <c r="D2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="N4" t="s">
         <v>324</v>
       </c>
-      <c r="F2" t="s">
+      <c r="O4" t="s">
         <v>325</v>
       </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="P4" t="s">
         <v>326</v>
       </c>
-      <c r="I2" t="s">
+      <c r="Q4" t="s">
         <v>327</v>
       </c>
-      <c r="J2" t="s">
+      <c r="R4" t="s">
+        <v>327</v>
+      </c>
+      <c r="S4" t="s">
         <v>328</v>
       </c>
-      <c r="K2" t="s">
+      <c r="T4" t="s">
         <v>329</v>
       </c>
-      <c r="L2" t="s">
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
         <v>330</v>
       </c>
-      <c r="M2" t="s">
-        <v>81</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="H5" t="s">
         <v>331</v>
       </c>
-      <c r="O2" t="s">
-        <v>81</v>
-      </c>
-      <c r="P2" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>83</v>
-      </c>
-      <c r="R2" t="s">
-        <v>55</v>
-      </c>
-      <c r="S2" t="s">
-        <v>84</v>
-      </c>
-      <c r="T2" t="s">
+      <c r="I5" t="s">
+        <v>330</v>
+      </c>
+      <c r="J5" t="s">
         <v>332</v>
       </c>
-      <c r="U2" t="s">
-        <v>85</v>
-      </c>
-      <c r="V2" t="s">
-        <v>86</v>
-      </c>
-      <c r="W2" t="s">
+      <c r="K5" t="s">
+        <v>72</v>
+      </c>
+      <c r="L5" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" t="s">
         <v>333</v>
       </c>
-      <c r="X2" t="s">
-        <v>333</v>
-      </c>
-      <c r="Y2" t="s">
+      <c r="N5" t="s">
         <v>334</v>
       </c>
-      <c r="Z2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M3" t="s">
+      <c r="O5" t="s">
         <v>335</v>
       </c>
-      <c r="N3" t="s">
+      <c r="P5" t="s">
         <v>336</v>
       </c>
-      <c r="O3" t="s">
-        <v>335</v>
-      </c>
-      <c r="P3" t="s">
+      <c r="Q5" t="s">
         <v>337</v>
       </c>
-      <c r="Q3" t="s">
-        <v>83</v>
-      </c>
-      <c r="R3" t="s">
-        <v>55</v>
-      </c>
-      <c r="S3" t="s">
+      <c r="R5" t="s">
+        <v>337</v>
+      </c>
+      <c r="S5" t="s">
         <v>338</v>
       </c>
-      <c r="T3" t="s">
+      <c r="T5" t="s">
         <v>339</v>
       </c>
-      <c r="U3" t="s">
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
         <v>340</v>
       </c>
-      <c r="V3" t="s">
+      <c r="H6" t="s">
         <v>341</v>
       </c>
-      <c r="W3" t="s">
+      <c r="I6" t="s">
+        <v>340</v>
+      </c>
+      <c r="J6" t="s">
         <v>342</v>
       </c>
-      <c r="X3" t="s">
-        <v>342</v>
-      </c>
-      <c r="Y3" t="s">
+      <c r="K6" t="s">
+        <v>72</v>
+      </c>
+      <c r="L6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M6" t="s">
         <v>343</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="N6" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M4" t="s">
+      <c r="O6" t="s">
         <v>345</v>
       </c>
-      <c r="N4" t="s">
+      <c r="P6" t="s">
         <v>346</v>
       </c>
-      <c r="O4" t="s">
-        <v>345</v>
-      </c>
-      <c r="P4" t="s">
+      <c r="Q6" t="s">
         <v>347</v>
       </c>
-      <c r="Q4" t="s">
-        <v>83</v>
-      </c>
-      <c r="R4" t="s">
-        <v>55</v>
-      </c>
-      <c r="S4" t="s">
+      <c r="R6" t="s">
+        <v>347</v>
+      </c>
+      <c r="S6" t="s">
         <v>348</v>
       </c>
-      <c r="T4" t="s">
+      <c r="T6" t="s">
         <v>349</v>
-      </c>
-      <c r="U4" t="s">
-        <v>350</v>
-      </c>
-      <c r="V4" t="s">
-        <v>351</v>
-      </c>
-      <c r="W4" t="s">
-        <v>352</v>
-      </c>
-      <c r="X4" t="s">
-        <v>352</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>353</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M5" t="s">
-        <v>355</v>
-      </c>
-      <c r="N5" t="s">
-        <v>356</v>
-      </c>
-      <c r="O5" t="s">
-        <v>355</v>
-      </c>
-      <c r="P5" t="s">
-        <v>357</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>83</v>
-      </c>
-      <c r="R5" t="s">
-        <v>55</v>
-      </c>
-      <c r="S5" t="s">
-        <v>358</v>
-      </c>
-      <c r="T5" t="s">
-        <v>359</v>
-      </c>
-      <c r="U5" t="s">
-        <v>360</v>
-      </c>
-      <c r="V5" t="s">
-        <v>361</v>
-      </c>
-      <c r="W5" t="s">
-        <v>362</v>
-      </c>
-      <c r="X5" t="s">
-        <v>362</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>363</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="M6" t="s">
-        <v>365</v>
-      </c>
-      <c r="N6" t="s">
-        <v>366</v>
-      </c>
-      <c r="O6" t="s">
-        <v>365</v>
-      </c>
-      <c r="P6" t="s">
-        <v>367</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>83</v>
-      </c>
-      <c r="R6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S6" t="s">
-        <v>368</v>
-      </c>
-      <c r="T6" t="s">
-        <v>369</v>
-      </c>
-      <c r="U6" t="s">
-        <v>370</v>
-      </c>
-      <c r="V6" t="s">
-        <v>371</v>
-      </c>
-      <c r="W6" t="s">
-        <v>372</v>
-      </c>
-      <c r="X6" t="s">
-        <v>372</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>373</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>374</v>
       </c>
     </row>
   </sheetData>
@@ -3691,337 +3451,337 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>102</v>
       </c>
       <c r="V1" s="1"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>407</v>
+        <v>382</v>
       </c>
       <c r="B2" t="s">
-        <v>408</v>
+        <v>383</v>
       </c>
       <c r="C2" t="s">
-        <v>409</v>
+        <v>384</v>
       </c>
       <c r="D2" t="s">
-        <v>410</v>
+        <v>385</v>
       </c>
       <c r="E2" t="s">
-        <v>411</v>
+        <v>386</v>
       </c>
       <c r="G2" t="s">
-        <v>412</v>
+        <v>387</v>
       </c>
       <c r="H2" t="s">
-        <v>413</v>
+        <v>388</v>
       </c>
       <c r="I2" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="J2" t="s">
-        <v>414</v>
+        <v>389</v>
       </c>
       <c r="K2" t="s">
-        <v>415</v>
+        <v>390</v>
       </c>
       <c r="L2" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="M2" t="s">
-        <v>416</v>
+        <v>391</v>
       </c>
       <c r="N2" t="s">
-        <v>417</v>
+        <v>392</v>
       </c>
       <c r="O2" t="s">
-        <v>418</v>
+        <v>393</v>
       </c>
       <c r="P2" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="Q2" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="R2" t="s">
-        <v>419</v>
+        <v>394</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="Q3" t="s">
-        <v>420</v>
+        <v>395</v>
       </c>
       <c r="R3" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="Q4" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="R4" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="Q5" t="s">
-        <v>422</v>
+        <v>397</v>
       </c>
       <c r="R5" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="L6" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="M6" t="s">
-        <v>423</v>
+        <v>398</v>
       </c>
       <c r="N6" t="s">
-        <v>424</v>
+        <v>399</v>
       </c>
       <c r="O6" t="s">
-        <v>418</v>
+        <v>393</v>
       </c>
       <c r="P6" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="Q6" t="s">
-        <v>352</v>
+        <v>327</v>
       </c>
       <c r="R6" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="Q7" t="s">
-        <v>425</v>
+        <v>400</v>
       </c>
       <c r="R7" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="Q8" t="s">
-        <v>426</v>
+        <v>401</v>
       </c>
       <c r="R8" t="s">
-        <v>419</v>
+        <v>394</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="Q9" t="s">
-        <v>427</v>
+        <v>402</v>
       </c>
       <c r="R9" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="L10" t="s">
-        <v>428</v>
+        <v>403</v>
       </c>
       <c r="M10" t="s">
-        <v>429</v>
+        <v>404</v>
       </c>
       <c r="N10" t="s">
-        <v>430</v>
+        <v>405</v>
       </c>
       <c r="O10" t="s">
-        <v>418</v>
+        <v>393</v>
       </c>
       <c r="P10" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="Q10" t="s">
-        <v>431</v>
+        <v>406</v>
       </c>
       <c r="R10" t="s">
-        <v>432</v>
+        <v>407</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="Q11" t="s">
-        <v>433</v>
+        <v>408</v>
       </c>
       <c r="R11" t="s">
-        <v>434</v>
+        <v>409</v>
       </c>
       <c r="S11" t="s">
-        <v>435</v>
+        <v>410</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="L12" t="s">
-        <v>436</v>
+        <v>411</v>
       </c>
       <c r="M12" t="s">
-        <v>437</v>
+        <v>412</v>
       </c>
       <c r="N12" t="s">
-        <v>438</v>
+        <v>413</v>
       </c>
       <c r="O12" t="s">
-        <v>418</v>
+        <v>393</v>
       </c>
       <c r="P12" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="Q12" t="s">
-        <v>439</v>
+        <v>414</v>
       </c>
       <c r="R12" t="s">
-        <v>440</v>
+        <v>415</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="Q13" t="s">
-        <v>441</v>
+        <v>416</v>
       </c>
       <c r="R13" t="s">
-        <v>442</v>
+        <v>417</v>
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="M14" t="s">
-        <v>437</v>
+        <v>412</v>
       </c>
       <c r="Q14" t="s">
-        <v>443</v>
+        <v>418</v>
       </c>
       <c r="R14" t="s">
-        <v>444</v>
+        <v>419</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="Q15" t="s">
-        <v>445</v>
+        <v>420</v>
       </c>
       <c r="R15" t="s">
-        <v>446</v>
+        <v>421</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="L16" t="s">
-        <v>447</v>
+        <v>422</v>
       </c>
       <c r="M16" t="s">
-        <v>448</v>
+        <v>423</v>
       </c>
       <c r="N16" t="s">
-        <v>449</v>
+        <v>424</v>
       </c>
       <c r="O16" t="s">
-        <v>418</v>
+        <v>393</v>
       </c>
       <c r="P16" t="s">
-        <v>450</v>
+        <v>425</v>
       </c>
       <c r="Q16" t="s">
-        <v>451</v>
+        <v>426</v>
       </c>
       <c r="R16" t="s">
-        <v>452</v>
+        <v>427</v>
       </c>
       <c r="S16" t="s">
-        <v>453</v>
+        <v>428</v>
       </c>
       <c r="T16" t="s">
-        <v>454</v>
+        <v>429</v>
       </c>
       <c r="U16" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
     </row>
     <row r="17" spans="17:21" x14ac:dyDescent="0.3">
       <c r="Q17" t="s">
-        <v>455</v>
+        <v>430</v>
       </c>
       <c r="S17" t="s">
-        <v>433</v>
+        <v>408</v>
       </c>
       <c r="T17" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="U17" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
     </row>
     <row r="18" spans="17:21" x14ac:dyDescent="0.3">
       <c r="S18" t="s">
-        <v>456</v>
+        <v>431</v>
       </c>
       <c r="T18" t="s">
-        <v>457</v>
+        <v>432</v>
       </c>
       <c r="U18" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
     </row>
     <row r="19" spans="17:21" x14ac:dyDescent="0.3">
       <c r="S19" t="s">
-        <v>458</v>
+        <v>433</v>
       </c>
       <c r="T19" t="s">
-        <v>459</v>
+        <v>434</v>
       </c>
       <c r="U19" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
     </row>
     <row r="20" spans="17:21" x14ac:dyDescent="0.3">
       <c r="S20" t="s">
-        <v>460</v>
+        <v>435</v>
       </c>
       <c r="T20" t="s">
-        <v>461</v>
+        <v>436</v>
       </c>
       <c r="U20" t="s">
-        <v>419</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add legacy header aliases for improved Excel import handling; update security config to remove package import endpoint from public access
</commit_message>
<xml_diff>
--- a/repo-learning-path/test-data/learning-path-import-full-test.xlsx
+++ b/repo-learning-path/test-data/learning-path-import-full-test.xlsx
@@ -2905,7 +2905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Definition</t>
+          <t>Meaning</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
@@ -2961,80 +2961,79 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
+          <t>OriginTextVi</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>OriginTextCn</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>OriginTextEn</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>OriginImage</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>AudioUrl</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>StrokeAnimationUrl</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>ExampleSentence</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>ExamplePinyin</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>ExampleMeaning</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>ExampleMeaningVi</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>ExampleMeaningEn</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
           <t>WordType</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>HskLevel</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>ImageWord</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>SinoOrigin</t>
-        </is>
-      </c>
-      <c r="O1" s="2" t="inlineStr">
-        <is>
-          <t>ImageOrigin</t>
-        </is>
-      </c>
-      <c r="P1" s="2" t="inlineStr">
-        <is>
-          <t>Audio</t>
-        </is>
-      </c>
-      <c r="Q1" s="2" t="inlineStr">
-        <is>
-          <t>ExampleSentence</t>
-        </is>
-      </c>
-      <c r="R1" s="2" t="inlineStr">
-        <is>
-          <t>ExamplePinyin</t>
-        </is>
-      </c>
-      <c r="S1" s="2" t="inlineStr">
-        <is>
-          <t>ExampleMeaning</t>
-        </is>
-      </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>CharactersJson</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
-        <is>
-          <t>OriginTextCn</t>
-        </is>
-      </c>
-      <c r="V1" s="2" t="inlineStr">
-        <is>
-          <t>OriginTextEn</t>
-        </is>
-      </c>
-      <c r="W1" s="2" t="inlineStr">
-        <is>
-          <t>StrokeAnimationUrl</t>
-        </is>
-      </c>
-      <c r="X1" s="2" t="inlineStr">
-        <is>
-          <t>ExampleMeaningVi</t>
-        </is>
-      </c>
-      <c r="Y1" s="2" t="inlineStr">
-        <is>
-          <t>ExampleMeaningEn</t>
-        </is>
-      </c>
-      <c r="Z1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3089,77 +3088,77 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>Chữ Nhật mô phỏng hình dáng mặt trời rực rỡ</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>日，象形字，表示太阳。</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>The character represents the sun</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>sun_origin.png</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>https://example.com/audio/ri.mp3</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>https://example.com/stroke/ri.gif</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>今天是生日</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>jīn tiān shì shēng rì</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Hôm nay là sinh nhật</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Hôm nay là sinh nhật</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Today is birthday</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
           <t>KANJI</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>HSK1</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>Hình ảnh mặt trời tròn có dấu chấm ở giữa</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Chữ Nhật mô phỏng hình dáng mặt trời rực rỡ</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>sun_origin.png</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>https://example.com/audio/ri.mp3</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>今天是生日</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>jīn tiān shì shēng rì</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Hôm nay là sinh nhật</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>[{"char":"日"}]</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>日，象形字，表示太阳。</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>The character represents the sun</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>https://example.com/stroke/ri.gif</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>Hôm nay là sinh nhật</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Today is birthday</t>
         </is>
       </c>
     </row>
@@ -3186,77 +3185,77 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>Mô phỏng hình ảnh mặt trăng lưỡi liềm</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>月，象形字，表示月亮。</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>The character represents the crescent moon</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>moon_origin.png</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>https://example.com/audio/yue.mp3</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>https://example.com/stroke/yue.gif</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>九月十号</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>jiǔ yuè shí hào</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Ngày 10 tháng 9</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Ngày 10 tháng 9</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>September 10th</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
           <t>KANJI</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>HSK1</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>Hình ảnh vầng trăng khuyết</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Mô phỏng hình ảnh mặt trăng lưỡi liềm</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>moon_origin.png</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>https://example.com/audio/yue.mp3</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>九月十号</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>jiǔ yuè shí hào</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Ngày 10 tháng 9</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>[{"char":"月"}]</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>月，象形字，表示月亮。</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>The character represents the crescent moon</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>https://example.com/stroke/yue.gif</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Ngày 10 tháng 9</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>September 10th</t>
         </is>
       </c>
     </row>
@@ -3283,77 +3282,77 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>Mô phỏng hình dáng các đỉnh núi cao</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>山，象形字，像山峰。</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>The character represents mountain peaks</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>mountain_origin.png</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>https://example.com/audio/shan.mp3</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>https://example.com/stroke/shan.gif</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>高山</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>gāo shān</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Núi cao</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Núi rất cao</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>High mountain</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
           <t>KANJI</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>HSK1</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>Hình ảnh ba đỉnh núi nhấp nhô</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Mô phỏng hình dáng các đỉnh núi cao</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>mountain_origin.png</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>https://example.com/audio/shan.mp3</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>高山</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>gāo shān</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Núi cao</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>[{"char":"山"}]</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>山，象形字，像山峰。</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>The character represents mountain peaks</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>https://example.com/stroke/shan.gif</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Núi rất cao</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>High mountain</t>
         </is>
       </c>
     </row>
@@ -3380,77 +3379,77 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>Mô phỏng dòng nước chảy ở giữa và tia nước hai bên</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>水，象形字，像流水。</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>The character represents flowing water</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>water_origin.png</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>https://example.com/audio/shui.mp3</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>https://example.com/stroke/shui.gif</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>喝水</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>hē shuǐ</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Uống nước</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Tôi muốn uống nước</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>I want to drink water</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
           <t>KANJI</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>HSK1</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>Hình ảnh dòng nước chảy cuộn</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Mô phỏng dòng nước chảy ở giữa và tia nước hai bên</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>water_origin.png</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>https://example.com/audio/shui.mp3</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>喝水</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>hē shuǐ</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Uống nước</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>[{"char":"水"}]</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>水，象形字，像流水。</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>The character represents flowing water</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>https://example.com/stroke/shui.gif</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>Tôi muốn uống nước</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>I want to drink water</t>
         </is>
       </c>
     </row>
@@ -3477,77 +3476,77 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>Mô phỏng đống lửa có các tia lửa bắn ra</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>火，象形字，像火焰。</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>The character represents a flickering flame</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>fire_origin.png</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>https://example.com/audio/huo.mp3</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>https://example.com/stroke/huo.gif</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>火车</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>huǒ chē</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Tàu hỏa</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Tàu hỏa chạy nhanh</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>The train runs fast</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
           <t>KANJI</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>HSK1</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>Hình ảnh ngọn lửa đang bốc cháy</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Mô phỏng đống lửa có các tia lửa bắn ra</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>fire_origin.png</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>https://example.com/audio/huo.mp3</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>火车</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>huǒ chē</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>Tàu hỏa</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>[{"char":"火"}]</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>火，象形字，像火焰。</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>The character represents a flickering flame</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>https://example.com/stroke/huo.gif</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>Tàu hỏa chạy nhanh</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>The train runs fast</t>
         </is>
       </c>
     </row>

</xml_diff>